<commit_message>
Release BTG Audit v12.0.0
</commit_message>
<xml_diff>
--- a/vendor_matrix_detailed.xlsx
+++ b/vendor_matrix_detailed.xlsx
@@ -2,16 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Matrix" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -21,17 +16,15 @@
   <fonts count="3">
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b val="1"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
   <fills count="6">
@@ -43,33 +36,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9EAD3"/>
+        <fgColor rgb="FFD9EAD3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
+        <fgColor rgb="FFF4CCCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -94,9 +81,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -280,72 +266,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -401,7 +329,7 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -410,13 +338,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -450,17 +378,6 @@
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -515,8 +432,6 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -526,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU31"/>
+  <dimension ref="A1:AY44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -696,120 +611,140 @@
       </c>
       <c r="X1" s="2" t="inlineStr">
         <is>
+          <t>IDS/IPS</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
           <t>WAF</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>SAST</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>DAST</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>SCA</t>
+        </is>
+      </c>
+      <c r="AC1" s="2" t="inlineStr">
         <is>
           <t>Anti-DDoS</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="AD1" s="2" t="inlineStr">
         <is>
           <t>ZTNA</t>
         </is>
       </c>
-      <c r="AA1" s="2" t="inlineStr">
+      <c r="AE1" s="2" t="inlineStr">
         <is>
           <t>SASE</t>
         </is>
       </c>
-      <c r="AB1" s="2" t="inlineStr">
+      <c r="AF1" s="2" t="inlineStr">
         <is>
           <t>NAC</t>
         </is>
       </c>
-      <c r="AC1" s="2" t="inlineStr">
+      <c r="AG1" s="2" t="inlineStr">
         <is>
           <t>MDM/UEM</t>
         </is>
       </c>
-      <c r="AD1" s="2" t="inlineStr">
+      <c r="AH1" s="2" t="inlineStr">
         <is>
           <t>MDR</t>
         </is>
       </c>
-      <c r="AE1" s="2" t="inlineStr">
+      <c r="AI1" s="2" t="inlineStr">
         <is>
           <t>IoT Security</t>
         </is>
       </c>
-      <c r="AF1" s="2" t="inlineStr">
+      <c r="AJ1" s="2" t="inlineStr">
         <is>
           <t>Network Equipment</t>
         </is>
       </c>
-      <c r="AG1" s="2" t="inlineStr">
+      <c r="AK1" s="2" t="inlineStr">
         <is>
           <t>Servers</t>
         </is>
       </c>
-      <c r="AH1" s="2" t="inlineStr">
+      <c r="AL1" s="2" t="inlineStr">
         <is>
           <t>Storage</t>
         </is>
       </c>
-      <c r="AI1" s="2" t="inlineStr">
+      <c r="AM1" s="2" t="inlineStr">
         <is>
           <t>Operating Systems</t>
         </is>
       </c>
-      <c r="AJ1" s="2" t="inlineStr">
+      <c r="AN1" s="2" t="inlineStr">
         <is>
           <t>Corporate Email</t>
         </is>
       </c>
-      <c r="AK1" s="2" t="inlineStr">
+      <c r="AO1" s="2" t="inlineStr">
         <is>
           <t>Virtualization</t>
         </is>
       </c>
-      <c r="AL1" s="2" t="inlineStr">
+      <c r="AP1" s="2" t="inlineStr">
         <is>
           <t>ITSM</t>
         </is>
       </c>
-      <c r="AM1" s="2" t="inlineStr">
+      <c r="AQ1" s="2" t="inlineStr">
         <is>
           <t>Patch Management</t>
         </is>
       </c>
-      <c r="AN1" s="2" t="inlineStr">
+      <c r="AR1" s="2" t="inlineStr">
         <is>
           <t>ITAM</t>
         </is>
       </c>
-      <c r="AO1" s="2" t="inlineStr">
+      <c r="AS1" s="2" t="inlineStr">
         <is>
           <t>Remote Access</t>
         </is>
       </c>
-      <c r="AP1" s="2" t="inlineStr">
+      <c r="AT1" s="2" t="inlineStr">
         <is>
           <t>Session Management</t>
         </is>
       </c>
-      <c r="AQ1" s="2" t="inlineStr">
+      <c r="AU1" s="2" t="inlineStr">
         <is>
           <t>Cloud Platform</t>
         </is>
       </c>
-      <c r="AR1" s="2" t="inlineStr">
+      <c r="AV1" s="2" t="inlineStr">
         <is>
           <t>Distributor KZ</t>
         </is>
       </c>
-      <c r="AS1" s="2" t="inlineStr">
+      <c r="AW1" s="2" t="inlineStr">
         <is>
           <t>Distributor Source</t>
         </is>
       </c>
-      <c r="AT1" s="2" t="inlineStr">
+      <c r="AX1" s="2" t="inlineStr">
         <is>
           <t>Distributor Status</t>
         </is>
       </c>
-      <c r="AU1" s="2" t="inlineStr">
+      <c r="AY1" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -889,32 +824,36 @@
       <c r="AI2" s="3" t="n"/>
       <c r="AJ2" s="3" t="n"/>
       <c r="AK2" s="3" t="n"/>
-      <c r="AL2" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AL2" s="3" t="n"/>
       <c r="AM2" s="3" t="n"/>
       <c r="AN2" s="3" t="n"/>
       <c r="AO2" s="3" t="n"/>
-      <c r="AP2" s="3" t="n"/>
+      <c r="AP2" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AQ2" s="3" t="n"/>
-      <c r="AR2" s="3" t="inlineStr">
+      <c r="AR2" s="3" t="n"/>
+      <c r="AS2" s="3" t="n"/>
+      <c r="AT2" s="3" t="n"/>
+      <c r="AU2" s="3" t="n"/>
+      <c r="AV2" s="3" t="inlineStr">
         <is>
           <t>MONT TECH; MUK</t>
         </is>
       </c>
-      <c r="AS2" s="3" t="inlineStr">
+      <c r="AW2" s="3" t="inlineStr">
         <is>
           <t>https://monttech.kz/ru-kz/vendors/symantec ; https://muk.group/ru/country/kz/</t>
         </is>
       </c>
-      <c r="AT2" s="4" t="inlineStr">
+      <c r="AX2" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU2" s="3" t="inlineStr"/>
+      <c r="AY2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -960,7 +899,11 @@
           <t>+</t>
         </is>
       </c>
-      <c r="X3" s="3" t="n"/>
+      <c r="X3" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="Y3" s="3" t="n"/>
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="3" t="n"/>
@@ -980,22 +923,26 @@
       <c r="AO3" s="3" t="n"/>
       <c r="AP3" s="3" t="n"/>
       <c r="AQ3" s="3" t="n"/>
-      <c r="AR3" s="3" t="inlineStr">
+      <c r="AR3" s="3" t="n"/>
+      <c r="AS3" s="3" t="n"/>
+      <c r="AT3" s="3" t="n"/>
+      <c r="AU3" s="3" t="n"/>
+      <c r="AV3" s="3" t="inlineStr">
         <is>
           <t>Softprom</t>
         </is>
       </c>
-      <c r="AS3" s="3" t="inlineStr">
+      <c r="AW3" s="3" t="inlineStr">
         <is>
           <t>https://softprom.com/vendor/forcepoint</t>
         </is>
       </c>
-      <c r="AT3" s="4" t="inlineStr">
+      <c r="AX3" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU3" s="3" t="inlineStr"/>
+      <c r="AY3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1049,22 +996,26 @@
       <c r="AO4" s="3" t="n"/>
       <c r="AP4" s="3" t="n"/>
       <c r="AQ4" s="3" t="n"/>
-      <c r="AR4" s="3" t="inlineStr">
+      <c r="AR4" s="3" t="n"/>
+      <c r="AS4" s="3" t="n"/>
+      <c r="AT4" s="3" t="n"/>
+      <c r="AU4" s="3" t="n"/>
+      <c r="AV4" s="3" t="inlineStr">
         <is>
           <t>MSMAX; Cyber-Soft (поставщики/интеграторы)</t>
         </is>
       </c>
-      <c r="AS4" s="3" t="inlineStr">
+      <c r="AW4" s="3" t="inlineStr">
         <is>
           <t>https://zecurion.com/channel-partners/locate-an-authorized-partner/ ; https://msmax.kz/katalog/dlp_zecurion/ ; https://cyber-soft.kz/zecurion/</t>
         </is>
       </c>
-      <c r="AT4" s="5" t="inlineStr">
+      <c r="AX4" s="5" t="inlineStr">
         <is>
           <t>Требует проверки</t>
         </is>
       </c>
-      <c r="AU4" s="3" t="inlineStr">
+      <c r="AY4" s="3" t="inlineStr">
         <is>
           <t>Официальный KZ-дистрибьютор в открытых источниках не найден; указаны найденные поставщики/каналы.</t>
         </is>
@@ -1130,18 +1081,22 @@
       <c r="AO5" s="3" t="n"/>
       <c r="AP5" s="3" t="n"/>
       <c r="AQ5" s="3" t="n"/>
-      <c r="AR5" s="3" t="inlineStr">
+      <c r="AR5" s="3" t="n"/>
+      <c r="AS5" s="3" t="n"/>
+      <c r="AT5" s="3" t="n"/>
+      <c r="AU5" s="3" t="n"/>
+      <c r="AV5" s="3" t="inlineStr">
         <is>
           <t>Не найдено в открытых источниках</t>
         </is>
       </c>
-      <c r="AS5" s="3" t="inlineStr"/>
-      <c r="AT5" s="5" t="inlineStr">
+      <c r="AW5" s="3" t="inlineStr"/>
+      <c r="AX5" s="5" t="inlineStr">
         <is>
           <t>Требует проверки</t>
         </is>
       </c>
-      <c r="AU5" s="3" t="inlineStr">
+      <c r="AY5" s="3" t="inlineStr">
         <is>
           <t>Нужна ручная проверка у вендора/локального представителя.</t>
         </is>
@@ -1162,11 +1117,7 @@
           <t>+</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="3" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
@@ -1196,53 +1147,57 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="3" t="n"/>
       <c r="AB6" s="3" t="n"/>
-      <c r="AC6" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AC6" s="3" t="n"/>
       <c r="AD6" s="3" t="n"/>
       <c r="AE6" s="3" t="n"/>
       <c r="AF6" s="3" t="n"/>
-      <c r="AG6" s="3" t="n"/>
+      <c r="AG6" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AH6" s="3" t="n"/>
       <c r="AI6" s="3" t="n"/>
       <c r="AJ6" s="3" t="n"/>
       <c r="AK6" s="3" t="n"/>
-      <c r="AL6" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AM6" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AN6" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AL6" s="3" t="n"/>
+      <c r="AM6" s="3" t="n"/>
+      <c r="AN6" s="3" t="n"/>
       <c r="AO6" s="3" t="n"/>
-      <c r="AP6" s="3" t="n"/>
-      <c r="AQ6" s="3" t="n"/>
+      <c r="AP6" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AQ6" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AR6" s="3" t="inlineStr">
         <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AS6" s="3" t="n"/>
+      <c r="AT6" s="3" t="n"/>
+      <c r="AU6" s="3" t="n"/>
+      <c r="AV6" s="3" t="inlineStr">
+        <is>
           <t>Syssoft Kazakhstan</t>
         </is>
       </c>
-      <c r="AS6" s="3" t="inlineStr">
+      <c r="AW6" s="3" t="inlineStr">
         <is>
           <t>https://www.syssoft-group.kz/vendor/manageengine</t>
         </is>
       </c>
-      <c r="AT6" s="6" t="inlineStr">
+      <c r="AX6" s="6" t="inlineStr">
         <is>
           <t>Канал/партнер</t>
         </is>
       </c>
-      <c r="AU6" s="3" t="inlineStr">
+      <c r="AY6" s="3" t="inlineStr">
         <is>
           <t>Подтверждена поставка/канал продаж; статус официального дистрибьютора отдельно не указан.</t>
         </is>
@@ -1300,22 +1255,26 @@
       <c r="AO7" s="3" t="n"/>
       <c r="AP7" s="3" t="n"/>
       <c r="AQ7" s="3" t="n"/>
-      <c r="AR7" s="3" t="inlineStr">
+      <c r="AR7" s="3" t="n"/>
+      <c r="AS7" s="3" t="n"/>
+      <c r="AT7" s="3" t="n"/>
+      <c r="AU7" s="3" t="n"/>
+      <c r="AV7" s="3" t="inlineStr">
         <is>
           <t>Не найдено в открытых источниках; проверять через CyberArk Partner Finder</t>
         </is>
       </c>
-      <c r="AS7" s="3" t="inlineStr">
+      <c r="AW7" s="3" t="inlineStr">
         <is>
           <t>https://www.cyberark.com/partner-finder/</t>
         </is>
       </c>
-      <c r="AT7" s="5" t="inlineStr">
+      <c r="AX7" s="5" t="inlineStr">
         <is>
           <t>Требует проверки</t>
         </is>
       </c>
-      <c r="AU7" s="3" t="inlineStr"/>
+      <c r="AY7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1370,33 +1329,37 @@
       <c r="AL8" s="3" t="n"/>
       <c r="AM8" s="3" t="n"/>
       <c r="AN8" s="3" t="n"/>
-      <c r="AO8" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AP8" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AO8" s="3" t="n"/>
+      <c r="AP8" s="3" t="n"/>
       <c r="AQ8" s="3" t="n"/>
-      <c r="AR8" s="3" t="inlineStr">
+      <c r="AR8" s="3" t="n"/>
+      <c r="AS8" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AT8" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AU8" s="3" t="n"/>
+      <c r="AV8" s="3" t="inlineStr">
         <is>
           <t>ABRIS Kazakhstan</t>
         </is>
       </c>
-      <c r="AS8" s="3" t="inlineStr">
+      <c r="AW8" s="3" t="inlineStr">
         <is>
           <t>https://www.wallix.com/partners/partner-finder/</t>
         </is>
       </c>
-      <c r="AT8" s="4" t="inlineStr">
+      <c r="AX8" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU8" s="3" t="inlineStr">
+      <c r="AY8" s="3" t="inlineStr">
         <is>
           <t>WALLIX Partner Finder показывает ABRIS Kazakhstan как VAD.</t>
         </is>
@@ -1455,33 +1418,37 @@
       <c r="AL9" s="3" t="n"/>
       <c r="AM9" s="3" t="n"/>
       <c r="AN9" s="3" t="n"/>
-      <c r="AO9" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AP9" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AO9" s="3" t="n"/>
+      <c r="AP9" s="3" t="n"/>
       <c r="AQ9" s="3" t="n"/>
-      <c r="AR9" s="3" t="inlineStr">
+      <c r="AR9" s="3" t="n"/>
+      <c r="AS9" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AT9" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AU9" s="3" t="n"/>
+      <c r="AV9" s="3" t="inlineStr">
         <is>
           <t>Не найдено в открытых источниках; проверять через BeyondTrust Partner Directory</t>
         </is>
       </c>
-      <c r="AS9" s="3" t="inlineStr">
+      <c r="AW9" s="3" t="inlineStr">
         <is>
           <t>https://www.beyondtrust.com/partners/directory</t>
         </is>
       </c>
-      <c r="AT9" s="5" t="inlineStr">
+      <c r="AX9" s="5" t="inlineStr">
         <is>
           <t>Требует проверки</t>
         </is>
       </c>
-      <c r="AU9" s="3" t="inlineStr"/>
+      <c r="AY9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1535,22 +1502,26 @@
       <c r="AO10" s="3" t="n"/>
       <c r="AP10" s="3" t="n"/>
       <c r="AQ10" s="3" t="n"/>
-      <c r="AR10" s="3" t="inlineStr">
+      <c r="AR10" s="3" t="n"/>
+      <c r="AS10" s="3" t="n"/>
+      <c r="AT10" s="3" t="n"/>
+      <c r="AU10" s="3" t="n"/>
+      <c r="AV10" s="3" t="inlineStr">
         <is>
           <t>MONT TECH</t>
         </is>
       </c>
-      <c r="AS10" s="3" t="inlineStr">
+      <c r="AW10" s="3" t="inlineStr">
         <is>
           <t>https://monttech.kz/ru-kz/vendors/veeam</t>
         </is>
       </c>
-      <c r="AT10" s="4" t="inlineStr">
+      <c r="AX10" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU10" s="3" t="inlineStr"/>
+      <c r="AY10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1604,22 +1575,26 @@
       <c r="AO11" s="3" t="n"/>
       <c r="AP11" s="3" t="n"/>
       <c r="AQ11" s="3" t="n"/>
-      <c r="AR11" s="3" t="inlineStr">
+      <c r="AR11" s="3" t="n"/>
+      <c r="AS11" s="3" t="n"/>
+      <c r="AT11" s="3" t="n"/>
+      <c r="AU11" s="3" t="n"/>
+      <c r="AV11" s="3" t="inlineStr">
         <is>
           <t>MONT TECH; Marvel Kazakhstan</t>
         </is>
       </c>
-      <c r="AS11" s="3" t="inlineStr">
+      <c r="AW11" s="3" t="inlineStr">
         <is>
           <t>https://monttech.kz/ru-kz/vendors/commvault ; https://www.marvel.kz/catalog/vendors/commvault/</t>
         </is>
       </c>
-      <c r="AT11" s="4" t="inlineStr">
+      <c r="AX11" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU11" s="3" t="inlineStr"/>
+      <c r="AY11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1673,22 +1648,26 @@
       <c r="AO12" s="3" t="n"/>
       <c r="AP12" s="3" t="n"/>
       <c r="AQ12" s="3" t="n"/>
-      <c r="AR12" s="3" t="inlineStr">
+      <c r="AR12" s="3" t="n"/>
+      <c r="AS12" s="3" t="n"/>
+      <c r="AT12" s="3" t="n"/>
+      <c r="AU12" s="3" t="n"/>
+      <c r="AV12" s="3" t="inlineStr">
         <is>
           <t>MUK</t>
         </is>
       </c>
-      <c r="AS12" s="3" t="inlineStr">
+      <c r="AW12" s="3" t="inlineStr">
         <is>
           <t>https://muk.group/ru/country/kz/</t>
         </is>
       </c>
-      <c r="AT12" s="4" t="inlineStr">
+      <c r="AX12" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU12" s="3" t="inlineStr"/>
+      <c r="AY12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1725,7 +1704,11 @@
           <t>+</t>
         </is>
       </c>
-      <c r="S13" s="3" t="n"/>
+      <c r="S13" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="T13" s="3" t="inlineStr">
         <is>
           <t>+</t>
@@ -1752,27 +1735,31 @@
           <t>+</t>
         </is>
       </c>
-      <c r="Z13" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AA13" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="Z13" s="3" t="n"/>
+      <c r="AA13" s="3" t="n"/>
       <c r="AB13" s="3" t="n"/>
-      <c r="AC13" s="3" t="n"/>
+      <c r="AC13" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AD13" s="3" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="AE13" s="3" t="n"/>
+      <c r="AE13" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AF13" s="3" t="n"/>
       <c r="AG13" s="3" t="n"/>
-      <c r="AH13" s="3" t="n"/>
+      <c r="AH13" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AI13" s="3" t="n"/>
       <c r="AJ13" s="3" t="n"/>
       <c r="AK13" s="3" t="n"/>
@@ -1782,22 +1769,26 @@
       <c r="AO13" s="3" t="n"/>
       <c r="AP13" s="3" t="n"/>
       <c r="AQ13" s="3" t="n"/>
-      <c r="AR13" s="3" t="inlineStr">
+      <c r="AR13" s="3" t="n"/>
+      <c r="AS13" s="3" t="n"/>
+      <c r="AT13" s="3" t="n"/>
+      <c r="AU13" s="3" t="n"/>
+      <c r="AV13" s="3" t="inlineStr">
         <is>
           <t>MONT TECH; MUK</t>
         </is>
       </c>
-      <c r="AS13" s="3" t="inlineStr">
+      <c r="AW13" s="3" t="inlineStr">
         <is>
           <t>https://monttech.kz/ru-kz/vendors/checkpoint ; https://muk.group/ru/country/kz/</t>
         </is>
       </c>
-      <c r="AT13" s="4" t="inlineStr">
+      <c r="AX13" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU13" s="3" t="inlineStr"/>
+      <c r="AY13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1847,18 +1838,14 @@
           <t>+</t>
         </is>
       </c>
-      <c r="X14" s="3" t="n"/>
+      <c r="X14" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="Y14" s="3" t="n"/>
-      <c r="Z14" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AA14" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="Z14" s="3" t="n"/>
+      <c r="AA14" s="3" t="n"/>
       <c r="AB14" s="3" t="n"/>
       <c r="AC14" s="3" t="n"/>
       <c r="AD14" s="3" t="inlineStr">
@@ -1866,10 +1853,18 @@
           <t>+</t>
         </is>
       </c>
-      <c r="AE14" s="3" t="n"/>
+      <c r="AE14" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AF14" s="3" t="n"/>
       <c r="AG14" s="3" t="n"/>
-      <c r="AH14" s="3" t="n"/>
+      <c r="AH14" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AI14" s="3" t="n"/>
       <c r="AJ14" s="3" t="n"/>
       <c r="AK14" s="3" t="n"/>
@@ -1879,22 +1874,26 @@
       <c r="AO14" s="3" t="n"/>
       <c r="AP14" s="3" t="n"/>
       <c r="AQ14" s="3" t="n"/>
-      <c r="AR14" s="3" t="inlineStr">
+      <c r="AR14" s="3" t="n"/>
+      <c r="AS14" s="3" t="n"/>
+      <c r="AT14" s="3" t="n"/>
+      <c r="AU14" s="3" t="n"/>
+      <c r="AV14" s="3" t="inlineStr">
         <is>
           <t>MUK</t>
         </is>
       </c>
-      <c r="AS14" s="3" t="inlineStr">
+      <c r="AW14" s="3" t="inlineStr">
         <is>
           <t>https://muk.group/kz/vendor/paloalto/ ; https://muk.group/ru/country/kz/</t>
         </is>
       </c>
-      <c r="AT14" s="4" t="inlineStr">
+      <c r="AX14" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU14" s="3" t="inlineStr"/>
+      <c r="AY14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1907,7 +1906,11 @@
       <c r="D15" s="3" t="n"/>
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="3" t="n"/>
-      <c r="G15" s="3" t="n"/>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="H15" s="3" t="n"/>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
@@ -1936,27 +1939,39 @@
           <t>+</t>
         </is>
       </c>
-      <c r="X15" s="3" t="n"/>
-      <c r="Y15" s="3" t="n"/>
-      <c r="Z15" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AA15" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AB15" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AC15" s="3" t="n"/>
-      <c r="AD15" s="3" t="n"/>
-      <c r="AE15" s="3" t="n"/>
-      <c r="AF15" s="3" t="n"/>
+      <c r="X15" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="Y15" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="Z15" s="3" t="n"/>
+      <c r="AA15" s="3" t="n"/>
+      <c r="AB15" s="3" t="n"/>
+      <c r="AC15" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AD15" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AE15" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AF15" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AG15" s="3" t="n"/>
       <c r="AH15" s="3" t="n"/>
       <c r="AI15" s="3" t="n"/>
@@ -1968,24 +1983,28 @@
       <c r="AO15" s="3" t="n"/>
       <c r="AP15" s="3" t="n"/>
       <c r="AQ15" s="3" t="n"/>
-      <c r="AR15" s="3" t="inlineStr">
+      <c r="AR15" s="3" t="n"/>
+      <c r="AS15" s="3" t="n"/>
+      <c r="AT15" s="3" t="n"/>
+      <c r="AU15" s="3" t="n"/>
+      <c r="AV15" s="3" t="inlineStr">
         <is>
           <t>Softprom; MUK</t>
         </is>
       </c>
-      <c r="AS15" s="3" t="inlineStr">
-        <is>
-          <t>https://partnerportal.fortinet.com/directory/search?l=Uzbekistan ; https://muk.group/ru/country/kz/</t>
-        </is>
-      </c>
-      <c r="AT15" s="4" t="inlineStr">
+      <c r="AW15" s="3" t="inlineStr">
+        <is>
+          <t>https://softprom.com/ru/vendor/fortinet ; https://muk.group/ru/country/kz/</t>
+        </is>
+      </c>
+      <c r="AX15" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU15" s="3" t="inlineStr">
-        <is>
-          <t>Fortinet locator показывает TOO Softprom как Master Distributor; MUK KZ также указывает Fortinet в портфеле.</t>
+      <c r="AY15" s="3" t="inlineStr">
+        <is>
+          <t>Softprom прямо указывает статус официального дистрибьютора Fortinet в Казахстане; MUK также включает Fortinet в портфель Казахстана.</t>
         </is>
       </c>
     </row>
@@ -2045,22 +2064,26 @@
       <c r="AO16" s="3" t="n"/>
       <c r="AP16" s="3" t="n"/>
       <c r="AQ16" s="3" t="n"/>
-      <c r="AR16" s="3" t="inlineStr">
+      <c r="AR16" s="3" t="n"/>
+      <c r="AS16" s="3" t="n"/>
+      <c r="AT16" s="3" t="n"/>
+      <c r="AU16" s="3" t="n"/>
+      <c r="AV16" s="3" t="inlineStr">
         <is>
           <t>AIC; ADELINE (реселлеры/партнеры, не дистрибьюторы)</t>
         </is>
       </c>
-      <c r="AS16" s="3" t="inlineStr">
+      <c r="AW16" s="3" t="inlineStr">
         <is>
           <t>https://elioplus.com/asia-pacific/kazakhstan/channel-partners/splunk ; https://www.splunk.com/en_us/partners.html</t>
         </is>
       </c>
-      <c r="AT16" s="6" t="inlineStr">
+      <c r="AX16" s="6" t="inlineStr">
         <is>
           <t>Канал/партнер</t>
         </is>
       </c>
-      <c r="AU16" s="3" t="inlineStr">
+      <c r="AY16" s="3" t="inlineStr">
         <is>
           <t>Официальный KZ-дистрибьютор не подтвержден; указан канал партнеров.</t>
         </is>
@@ -2116,15 +2139,15 @@
       <c r="AA17" s="3" t="n"/>
       <c r="AB17" s="3" t="n"/>
       <c r="AC17" s="3" t="n"/>
-      <c r="AD17" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AD17" s="3" t="n"/>
       <c r="AE17" s="3" t="n"/>
       <c r="AF17" s="3" t="n"/>
       <c r="AG17" s="3" t="n"/>
-      <c r="AH17" s="3" t="n"/>
+      <c r="AH17" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AI17" s="3" t="n"/>
       <c r="AJ17" s="3" t="n"/>
       <c r="AK17" s="3" t="n"/>
@@ -2134,22 +2157,26 @@
       <c r="AO17" s="3" t="n"/>
       <c r="AP17" s="3" t="n"/>
       <c r="AQ17" s="3" t="n"/>
-      <c r="AR17" s="3" t="inlineStr">
+      <c r="AR17" s="3" t="n"/>
+      <c r="AS17" s="3" t="n"/>
+      <c r="AT17" s="3" t="n"/>
+      <c r="AU17" s="3" t="n"/>
+      <c r="AV17" s="3" t="inlineStr">
         <is>
           <t>Не найдено в открытых источниках; проверять через Rapid7 Partner Directory</t>
         </is>
       </c>
-      <c r="AS17" s="3" t="inlineStr">
+      <c r="AW17" s="3" t="inlineStr">
         <is>
           <t>https://www.rapid7.com/partners/partners-directory/</t>
         </is>
       </c>
-      <c r="AT17" s="5" t="inlineStr">
+      <c r="AX17" s="5" t="inlineStr">
         <is>
           <t>Требует проверки</t>
         </is>
       </c>
-      <c r="AU17" s="3" t="inlineStr"/>
+      <c r="AY17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -2192,16 +2219,8 @@
       <c r="AD18" s="3" t="n"/>
       <c r="AE18" s="3" t="n"/>
       <c r="AF18" s="3" t="n"/>
-      <c r="AG18" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AH18" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AG18" s="3" t="n"/>
+      <c r="AH18" s="3" t="n"/>
       <c r="AI18" s="3" t="n"/>
       <c r="AJ18" s="3" t="n"/>
       <c r="AK18" s="3" t="inlineStr">
@@ -2209,28 +2228,40 @@
           <t>+</t>
         </is>
       </c>
-      <c r="AL18" s="3" t="n"/>
+      <c r="AL18" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AM18" s="3" t="n"/>
       <c r="AN18" s="3" t="n"/>
-      <c r="AO18" s="3" t="n"/>
+      <c r="AO18" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AP18" s="3" t="n"/>
       <c r="AQ18" s="3" t="n"/>
-      <c r="AR18" s="3" t="inlineStr">
+      <c r="AR18" s="3" t="n"/>
+      <c r="AS18" s="3" t="n"/>
+      <c r="AT18" s="3" t="n"/>
+      <c r="AU18" s="3" t="n"/>
+      <c r="AV18" s="3" t="inlineStr">
         <is>
           <t>MUK</t>
         </is>
       </c>
-      <c r="AS18" s="3" t="inlineStr">
+      <c r="AW18" s="3" t="inlineStr">
         <is>
           <t>https://muk.group/ru/country/kz/</t>
         </is>
       </c>
-      <c r="AT18" s="4" t="inlineStr">
+      <c r="AX18" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU18" s="3" t="inlineStr"/>
+      <c r="AY18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -2269,53 +2300,57 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="3" t="n"/>
       <c r="AB19" s="3" t="n"/>
-      <c r="AC19" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AC19" s="3" t="n"/>
       <c r="AD19" s="3" t="n"/>
       <c r="AE19" s="3" t="n"/>
       <c r="AF19" s="3" t="n"/>
-      <c r="AG19" s="3" t="n"/>
+      <c r="AG19" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AH19" s="3" t="n"/>
       <c r="AI19" s="3" t="n"/>
       <c r="AJ19" s="3" t="n"/>
       <c r="AK19" s="3" t="n"/>
-      <c r="AL19" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AM19" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AN19" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AL19" s="3" t="n"/>
+      <c r="AM19" s="3" t="n"/>
+      <c r="AN19" s="3" t="n"/>
       <c r="AO19" s="3" t="n"/>
-      <c r="AP19" s="3" t="n"/>
-      <c r="AQ19" s="3" t="n"/>
+      <c r="AP19" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AQ19" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AR19" s="3" t="inlineStr">
         <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AS19" s="3" t="n"/>
+      <c r="AT19" s="3" t="n"/>
+      <c r="AU19" s="3" t="n"/>
+      <c r="AV19" s="3" t="inlineStr">
+        <is>
           <t>MUK</t>
         </is>
       </c>
-      <c r="AS19" s="3" t="inlineStr">
+      <c r="AW19" s="3" t="inlineStr">
         <is>
           <t>https://muk.group/ru/country/kz/</t>
         </is>
       </c>
-      <c r="AT19" s="4" t="inlineStr">
+      <c r="AX19" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU19" s="3" t="inlineStr"/>
+      <c r="AY19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -2328,7 +2363,11 @@
       <c r="D20" s="3" t="n"/>
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="H20" s="3" t="n"/>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
@@ -2356,47 +2395,51 @@
       <c r="AF20" s="3" t="n"/>
       <c r="AG20" s="3" t="n"/>
       <c r="AH20" s="3" t="n"/>
-      <c r="AI20" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AJ20" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AK20" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AI20" s="3" t="n"/>
+      <c r="AJ20" s="3" t="n"/>
+      <c r="AK20" s="3" t="n"/>
       <c r="AL20" s="3" t="n"/>
-      <c r="AM20" s="3" t="n"/>
-      <c r="AN20" s="3" t="n"/>
-      <c r="AO20" s="3" t="n"/>
+      <c r="AM20" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AN20" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AO20" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AP20" s="3" t="n"/>
-      <c r="AQ20" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AR20" s="3" t="inlineStr">
+      <c r="AQ20" s="3" t="n"/>
+      <c r="AR20" s="3" t="n"/>
+      <c r="AS20" s="3" t="n"/>
+      <c r="AT20" s="3" t="n"/>
+      <c r="AU20" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AV20" s="3" t="inlineStr">
         <is>
           <t>MUK Cloud / MUK CSP</t>
         </is>
       </c>
-      <c r="AS20" s="3" t="inlineStr">
+      <c r="AW20" s="3" t="inlineStr">
         <is>
           <t>https://muk.group/ru/country/kz/ ; https://b2bcloud.muk.kz/</t>
         </is>
       </c>
-      <c r="AT20" s="4" t="inlineStr">
+      <c r="AX20" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU20" s="3" t="inlineStr"/>
+      <c r="AY20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -2445,15 +2488,15 @@
       <c r="AB21" s="3" t="n"/>
       <c r="AC21" s="3" t="n"/>
       <c r="AD21" s="3" t="n"/>
-      <c r="AE21" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AE21" s="3" t="n"/>
       <c r="AF21" s="3" t="n"/>
       <c r="AG21" s="3" t="n"/>
       <c r="AH21" s="3" t="n"/>
-      <c r="AI21" s="3" t="n"/>
+      <c r="AI21" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AJ21" s="3" t="n"/>
       <c r="AK21" s="3" t="n"/>
       <c r="AL21" s="3" t="n"/>
@@ -2462,22 +2505,26 @@
       <c r="AO21" s="3" t="n"/>
       <c r="AP21" s="3" t="n"/>
       <c r="AQ21" s="3" t="n"/>
-      <c r="AR21" s="3" t="inlineStr">
+      <c r="AR21" s="3" t="n"/>
+      <c r="AS21" s="3" t="n"/>
+      <c r="AT21" s="3" t="n"/>
+      <c r="AU21" s="3" t="n"/>
+      <c r="AV21" s="3" t="inlineStr">
         <is>
           <t>MONT TECH; 1C Kazakhstan</t>
         </is>
       </c>
-      <c r="AS21" s="3" t="inlineStr">
+      <c r="AW21" s="3" t="inlineStr">
         <is>
           <t>https://monttech.kz/ru-kz/vendors/kaspersky ; https://dist.1c.kz/catalog/kaspersky/</t>
         </is>
       </c>
-      <c r="AT21" s="4" t="inlineStr">
+      <c r="AX21" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU21" s="3" t="inlineStr"/>
+      <c r="AY21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -2530,15 +2577,15 @@
       <c r="AB22" s="3" t="n"/>
       <c r="AC22" s="3" t="n"/>
       <c r="AD22" s="3" t="n"/>
-      <c r="AE22" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AE22" s="3" t="n"/>
       <c r="AF22" s="3" t="n"/>
       <c r="AG22" s="3" t="n"/>
       <c r="AH22" s="3" t="n"/>
-      <c r="AI22" s="3" t="n"/>
+      <c r="AI22" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AJ22" s="3" t="n"/>
       <c r="AK22" s="3" t="n"/>
       <c r="AL22" s="3" t="n"/>
@@ -2547,22 +2594,26 @@
       <c r="AO22" s="3" t="n"/>
       <c r="AP22" s="3" t="n"/>
       <c r="AQ22" s="3" t="n"/>
-      <c r="AR22" s="3" t="inlineStr">
+      <c r="AR22" s="3" t="n"/>
+      <c r="AS22" s="3" t="n"/>
+      <c r="AT22" s="3" t="n"/>
+      <c r="AU22" s="3" t="n"/>
+      <c r="AV22" s="3" t="inlineStr">
         <is>
           <t>MONT TECH</t>
         </is>
       </c>
-      <c r="AS22" s="3" t="inlineStr">
+      <c r="AW22" s="3" t="inlineStr">
         <is>
           <t>https://monttech.kz/ru-KZ/vendors/trendmicro</t>
         </is>
       </c>
-      <c r="AT22" s="4" t="inlineStr">
+      <c r="AX22" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU22" s="3" t="inlineStr"/>
+      <c r="AY22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -2618,15 +2669,15 @@
       <c r="AA23" s="3" t="n"/>
       <c r="AB23" s="3" t="n"/>
       <c r="AC23" s="3" t="n"/>
-      <c r="AD23" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AD23" s="3" t="n"/>
       <c r="AE23" s="3" t="n"/>
       <c r="AF23" s="3" t="n"/>
       <c r="AG23" s="3" t="n"/>
-      <c r="AH23" s="3" t="n"/>
+      <c r="AH23" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AI23" s="3" t="n"/>
       <c r="AJ23" s="3" t="n"/>
       <c r="AK23" s="3" t="n"/>
@@ -2636,22 +2687,26 @@
       <c r="AO23" s="3" t="n"/>
       <c r="AP23" s="3" t="n"/>
       <c r="AQ23" s="3" t="n"/>
-      <c r="AR23" s="3" t="inlineStr">
+      <c r="AR23" s="3" t="n"/>
+      <c r="AS23" s="3" t="n"/>
+      <c r="AT23" s="3" t="n"/>
+      <c r="AU23" s="3" t="n"/>
+      <c r="AV23" s="3" t="inlineStr">
         <is>
           <t>Softprom</t>
         </is>
       </c>
-      <c r="AS23" s="3" t="inlineStr">
+      <c r="AW23" s="3" t="inlineStr">
         <is>
           <t>https://softprom.com/ru/softprom-distribyutor-crowdstrike</t>
         </is>
       </c>
-      <c r="AT23" s="4" t="inlineStr">
+      <c r="AX23" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU23" s="3" t="inlineStr"/>
+      <c r="AY23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -2692,7 +2747,11 @@
       <c r="X24" s="3" t="n"/>
       <c r="Y24" s="3" t="n"/>
       <c r="Z24" s="3" t="n"/>
-      <c r="AA24" s="3" t="n"/>
+      <c r="AA24" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AB24" s="3" t="n"/>
       <c r="AC24" s="3" t="n"/>
       <c r="AD24" s="3" t="n"/>
@@ -2704,35 +2763,39 @@
       <c r="AJ24" s="3" t="n"/>
       <c r="AK24" s="3" t="n"/>
       <c r="AL24" s="3" t="n"/>
-      <c r="AM24" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AN24" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AM24" s="3" t="n"/>
+      <c r="AN24" s="3" t="n"/>
       <c r="AO24" s="3" t="n"/>
       <c r="AP24" s="3" t="n"/>
-      <c r="AQ24" s="3" t="n"/>
+      <c r="AQ24" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AR24" s="3" t="inlineStr">
         <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AS24" s="3" t="n"/>
+      <c r="AT24" s="3" t="n"/>
+      <c r="AU24" s="3" t="n"/>
+      <c r="AV24" s="3" t="inlineStr">
+        <is>
           <t>MONT TECH</t>
         </is>
       </c>
-      <c r="AS24" s="3" t="inlineStr">
+      <c r="AW24" s="3" t="inlineStr">
         <is>
           <t>https://monttech.kz/ru-kz/vendors/qualys</t>
         </is>
       </c>
-      <c r="AT24" s="4" t="inlineStr">
+      <c r="AX24" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU24" s="3" t="inlineStr"/>
+      <c r="AY24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -2790,22 +2853,30 @@
       <c r="AO25" s="3" t="n"/>
       <c r="AP25" s="3" t="n"/>
       <c r="AQ25" s="3" t="n"/>
-      <c r="AR25" s="3" t="inlineStr">
-        <is>
-          <t>BAKOTECH; ATYPE KFT</t>
-        </is>
-      </c>
-      <c r="AS25" s="3" t="inlineStr">
-        <is>
-          <t>https://www.tenable.com/partner-locator/distributors ; https://bakotech.com/ru-kz/vendor/tenable/</t>
-        </is>
-      </c>
-      <c r="AT25" s="4" t="inlineStr">
+      <c r="AR25" s="3" t="n"/>
+      <c r="AS25" s="3" t="n"/>
+      <c r="AT25" s="3" t="n"/>
+      <c r="AU25" s="3" t="n"/>
+      <c r="AV25" s="3" t="inlineStr">
+        <is>
+          <t>BAKOTECH</t>
+        </is>
+      </c>
+      <c r="AW25" s="3" t="inlineStr">
+        <is>
+          <t>https://bakotech.com/ru-kz/vendor/tenable/ ; https://tenable.bakotech.com/home-en</t>
+        </is>
+      </c>
+      <c r="AX25" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU25" s="3" t="inlineStr"/>
+      <c r="AY25" s="3" t="inlineStr">
+        <is>
+          <t>BAKOTECH подтверждает официальный дистрибьюторский статус Tenable в Казахстане и Центральной Азии.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -2818,7 +2889,11 @@
       <c r="D26" s="3" t="n"/>
       <c r="E26" s="3" t="n"/>
       <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="H26" s="3" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
@@ -2835,15 +2910,15 @@
       <c r="U26" s="3" t="n"/>
       <c r="V26" s="3" t="n"/>
       <c r="W26" s="3" t="n"/>
-      <c r="X26" s="3" t="n"/>
+      <c r="X26" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="Y26" s="3" t="n"/>
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="3" t="n"/>
-      <c r="AB26" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AB26" s="3" t="n"/>
       <c r="AC26" s="3" t="n"/>
       <c r="AD26" s="3" t="n"/>
       <c r="AE26" s="3" t="n"/>
@@ -2855,7 +2930,11 @@
       <c r="AG26" s="3" t="n"/>
       <c r="AH26" s="3" t="n"/>
       <c r="AI26" s="3" t="n"/>
-      <c r="AJ26" s="3" t="n"/>
+      <c r="AJ26" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AK26" s="3" t="n"/>
       <c r="AL26" s="3" t="n"/>
       <c r="AM26" s="3" t="n"/>
@@ -2863,22 +2942,30 @@
       <c r="AO26" s="3" t="n"/>
       <c r="AP26" s="3" t="n"/>
       <c r="AQ26" s="3" t="n"/>
-      <c r="AR26" s="3" t="inlineStr">
-        <is>
-          <t>MUK; Marvel Kazakhstan; Isoft Kazakhstan</t>
-        </is>
-      </c>
-      <c r="AS26" s="3" t="inlineStr">
-        <is>
-          <t>https://muk.group/kz/vendor/cisco/ ; https://www.ciscochannelconnect.com/DistiProfile/182 ; https://isoft-shop.kz/cisco</t>
-        </is>
-      </c>
-      <c r="AT26" s="4" t="inlineStr">
+      <c r="AR26" s="3" t="n"/>
+      <c r="AS26" s="3" t="n"/>
+      <c r="AT26" s="3" t="n"/>
+      <c r="AU26" s="3" t="n"/>
+      <c r="AV26" s="3" t="inlineStr">
+        <is>
+          <t>Marvel Kazakhstan</t>
+        </is>
+      </c>
+      <c r="AW26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ciscochannelconnect.com/DistiProfile/182</t>
+        </is>
+      </c>
+      <c r="AX26" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU26" s="3" t="inlineStr"/>
+      <c r="AY26" s="3" t="inlineStr">
+        <is>
+          <t>Cisco Channel Connect указывает Marvel Kazakhstan как аккредитованного дистрибьютора Cisco в Алматы.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -2916,42 +3003,50 @@
       <c r="AC27" s="3" t="n"/>
       <c r="AD27" s="3" t="n"/>
       <c r="AE27" s="3" t="n"/>
-      <c r="AF27" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AG27" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AF27" s="3" t="n"/>
+      <c r="AG27" s="3" t="n"/>
       <c r="AH27" s="3" t="n"/>
       <c r="AI27" s="3" t="n"/>
-      <c r="AJ27" s="3" t="n"/>
-      <c r="AK27" s="3" t="n"/>
+      <c r="AJ27" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AK27" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AL27" s="3" t="n"/>
       <c r="AM27" s="3" t="n"/>
       <c r="AN27" s="3" t="n"/>
       <c r="AO27" s="3" t="n"/>
       <c r="AP27" s="3" t="n"/>
       <c r="AQ27" s="3" t="n"/>
-      <c r="AR27" s="3" t="inlineStr">
-        <is>
-          <t>ATACOM; MUK</t>
-        </is>
-      </c>
-      <c r="AS27" s="3" t="inlineStr">
-        <is>
-          <t>https://atacom.kz/en/ ; https://muk.group/ru/country/kz/</t>
-        </is>
-      </c>
-      <c r="AT27" s="4" t="inlineStr">
+      <c r="AR27" s="3" t="n"/>
+      <c r="AS27" s="3" t="n"/>
+      <c r="AT27" s="3" t="n"/>
+      <c r="AU27" s="3" t="n"/>
+      <c r="AV27" s="3" t="inlineStr">
+        <is>
+          <t>ATACOM</t>
+        </is>
+      </c>
+      <c r="AW27" s="3" t="inlineStr">
+        <is>
+          <t>https://atacom.kz/</t>
+        </is>
+      </c>
+      <c r="AX27" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU27" s="3" t="inlineStr"/>
+      <c r="AY27" s="3" t="inlineStr">
+        <is>
+          <t>ATACOM прямо указывает статус официального дистрибьютора Huawei в Республике Казахстан.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -2989,15 +3084,15 @@
       <c r="AC28" s="3" t="n"/>
       <c r="AD28" s="3" t="n"/>
       <c r="AE28" s="3" t="n"/>
-      <c r="AF28" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AF28" s="3" t="n"/>
       <c r="AG28" s="3" t="n"/>
       <c r="AH28" s="3" t="n"/>
       <c r="AI28" s="3" t="n"/>
-      <c r="AJ28" s="3" t="n"/>
+      <c r="AJ28" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AK28" s="3" t="n"/>
       <c r="AL28" s="3" t="n"/>
       <c r="AM28" s="3" t="n"/>
@@ -3005,22 +3100,26 @@
       <c r="AO28" s="3" t="n"/>
       <c r="AP28" s="3" t="n"/>
       <c r="AQ28" s="3" t="n"/>
-      <c r="AR28" s="3" t="inlineStr">
+      <c r="AR28" s="3" t="n"/>
+      <c r="AS28" s="3" t="n"/>
+      <c r="AT28" s="3" t="n"/>
+      <c r="AU28" s="3" t="n"/>
+      <c r="AV28" s="3" t="inlineStr">
         <is>
           <t>ATACOM</t>
         </is>
       </c>
-      <c r="AS28" s="3" t="inlineStr">
+      <c r="AW28" s="3" t="inlineStr">
         <is>
           <t>https://atacom.kz/en/</t>
         </is>
       </c>
-      <c r="AT28" s="4" t="inlineStr">
+      <c r="AX28" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU28" s="3" t="inlineStr"/>
+      <c r="AY28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -3058,15 +3157,15 @@
       <c r="AC29" s="3" t="n"/>
       <c r="AD29" s="3" t="n"/>
       <c r="AE29" s="3" t="n"/>
-      <c r="AF29" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AF29" s="3" t="n"/>
       <c r="AG29" s="3" t="n"/>
       <c r="AH29" s="3" t="n"/>
       <c r="AI29" s="3" t="n"/>
-      <c r="AJ29" s="3" t="n"/>
+      <c r="AJ29" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AK29" s="3" t="n"/>
       <c r="AL29" s="3" t="n"/>
       <c r="AM29" s="3" t="n"/>
@@ -3074,18 +3173,22 @@
       <c r="AO29" s="3" t="n"/>
       <c r="AP29" s="3" t="n"/>
       <c r="AQ29" s="3" t="n"/>
-      <c r="AR29" s="3" t="inlineStr">
+      <c r="AR29" s="3" t="n"/>
+      <c r="AS29" s="3" t="n"/>
+      <c r="AT29" s="3" t="n"/>
+      <c r="AU29" s="3" t="n"/>
+      <c r="AV29" s="3" t="inlineStr">
         <is>
           <t>Не найдено надежного подтверждения</t>
         </is>
       </c>
-      <c r="AS29" s="3" t="inlineStr"/>
-      <c r="AT29" s="5" t="inlineStr">
+      <c r="AW29" s="3" t="inlineStr"/>
+      <c r="AX29" s="5" t="inlineStr">
         <is>
           <t>Требует проверки</t>
         </is>
       </c>
-      <c r="AU29" s="3" t="inlineStr"/>
+      <c r="AY29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -3124,37 +3227,45 @@
       <c r="AD30" s="3" t="n"/>
       <c r="AE30" s="3" t="n"/>
       <c r="AF30" s="3" t="n"/>
-      <c r="AG30" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AG30" s="3" t="n"/>
       <c r="AH30" s="3" t="n"/>
       <c r="AI30" s="3" t="n"/>
       <c r="AJ30" s="3" t="n"/>
-      <c r="AK30" s="3" t="n"/>
+      <c r="AK30" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AL30" s="3" t="n"/>
       <c r="AM30" s="3" t="n"/>
       <c r="AN30" s="3" t="n"/>
       <c r="AO30" s="3" t="n"/>
       <c r="AP30" s="3" t="n"/>
       <c r="AQ30" s="3" t="n"/>
-      <c r="AR30" s="3" t="inlineStr">
-        <is>
-          <t>Techpro DC; Marvel Kazakhstan; MUK</t>
-        </is>
-      </c>
-      <c r="AS30" s="3" t="inlineStr">
-        <is>
-          <t>https://techprodc.com/ ; https://www.marvel.kz/ ; https://muk.group/ru/country/kz/</t>
-        </is>
-      </c>
-      <c r="AT30" s="4" t="inlineStr">
+      <c r="AR30" s="3" t="n"/>
+      <c r="AS30" s="3" t="n"/>
+      <c r="AT30" s="3" t="n"/>
+      <c r="AU30" s="3" t="n"/>
+      <c r="AV30" s="3" t="inlineStr">
+        <is>
+          <t>Marvel Kazakhstan</t>
+        </is>
+      </c>
+      <c r="AW30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.marvel.kz/press/news/?vendor=458 ; https://www.marvel.kz/catalog/vendors/hpe/</t>
+        </is>
+      </c>
+      <c r="AX30" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU30" s="3" t="inlineStr"/>
+      <c r="AY30" s="3" t="inlineStr">
+        <is>
+          <t>Marvel Kazakhstan подтверждает действующую дистрибуцию HP/HPE в Казахстане; убраны неподтвержденные текущими источниками записи.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -3193,40 +3304,1060 @@
       <c r="AD31" s="3" t="n"/>
       <c r="AE31" s="3" t="n"/>
       <c r="AF31" s="3" t="n"/>
-      <c r="AG31" s="3" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
+      <c r="AG31" s="3" t="n"/>
       <c r="AH31" s="3" t="n"/>
       <c r="AI31" s="3" t="n"/>
       <c r="AJ31" s="3" t="n"/>
-      <c r="AK31" s="3" t="n"/>
+      <c r="AK31" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AL31" s="3" t="n"/>
       <c r="AM31" s="3" t="n"/>
       <c r="AN31" s="3" t="n"/>
       <c r="AO31" s="3" t="n"/>
       <c r="AP31" s="3" t="n"/>
       <c r="AQ31" s="3" t="n"/>
-      <c r="AR31" s="3" t="inlineStr">
-        <is>
-          <t>MUK; Techpro DC</t>
-        </is>
-      </c>
-      <c r="AS31" s="3" t="inlineStr">
-        <is>
-          <t>https://muk.group/ru/country/kz/ ; https://techprodc.com/</t>
-        </is>
-      </c>
-      <c r="AT31" s="4" t="inlineStr">
+      <c r="AR31" s="3" t="n"/>
+      <c r="AS31" s="3" t="n"/>
+      <c r="AT31" s="3" t="n"/>
+      <c r="AU31" s="3" t="n"/>
+      <c r="AV31" s="3" t="inlineStr">
+        <is>
+          <t>MUK</t>
+        </is>
+      </c>
+      <c r="AW31" s="3" t="inlineStr">
+        <is>
+          <t>https://muk.group/ru/country/kz/ ; https://muk.group/rs/vendor/dell/</t>
+        </is>
+      </c>
+      <c r="AX31" s="4" t="inlineStr">
         <is>
           <t>Подтверждено</t>
         </is>
       </c>
-      <c r="AU31" s="3" t="inlineStr"/>
+      <c r="AY31" s="3" t="inlineStr">
+        <is>
+          <t>MUK указывает Dell Technologies в дистрибьюторском портфеле Казахстана и имеет статус Authorized Distributor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n"/>
+      <c r="C32" s="3" t="n"/>
+      <c r="D32" s="3" t="n"/>
+      <c r="E32" s="3" t="n"/>
+      <c r="F32" s="3" t="n"/>
+      <c r="G32" s="3" t="n"/>
+      <c r="H32" s="3" t="n"/>
+      <c r="I32" s="3" t="n"/>
+      <c r="J32" s="3" t="n"/>
+      <c r="K32" s="3" t="n"/>
+      <c r="L32" s="3" t="n"/>
+      <c r="M32" s="3" t="n"/>
+      <c r="N32" s="3" t="n"/>
+      <c r="O32" s="3" t="n"/>
+      <c r="P32" s="3" t="n"/>
+      <c r="Q32" s="3" t="n"/>
+      <c r="R32" s="3" t="n"/>
+      <c r="S32" s="3" t="n"/>
+      <c r="T32" s="3" t="n"/>
+      <c r="U32" s="3" t="n"/>
+      <c r="V32" s="3" t="n"/>
+      <c r="W32" s="3" t="n"/>
+      <c r="X32" s="3" t="n"/>
+      <c r="Y32" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="Z32" s="3" t="n"/>
+      <c r="AA32" s="3" t="n"/>
+      <c r="AB32" s="3" t="n"/>
+      <c r="AC32" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AD32" s="3" t="n"/>
+      <c r="AE32" s="3" t="n"/>
+      <c r="AF32" s="3" t="n"/>
+      <c r="AG32" s="3" t="n"/>
+      <c r="AH32" s="3" t="n"/>
+      <c r="AI32" s="3" t="n"/>
+      <c r="AJ32" s="3" t="n"/>
+      <c r="AK32" s="3" t="n"/>
+      <c r="AL32" s="3" t="n"/>
+      <c r="AM32" s="3" t="n"/>
+      <c r="AN32" s="3" t="n"/>
+      <c r="AO32" s="3" t="n"/>
+      <c r="AP32" s="3" t="n"/>
+      <c r="AQ32" s="3" t="n"/>
+      <c r="AR32" s="3" t="n"/>
+      <c r="AS32" s="3" t="n"/>
+      <c r="AT32" s="3" t="n"/>
+      <c r="AU32" s="3" t="n"/>
+      <c r="AV32" s="3" t="inlineStr">
+        <is>
+          <t>Не подтверждено; проверить через partner locator</t>
+        </is>
+      </c>
+      <c r="AW32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.f5.com/partners/find-a-partner</t>
+        </is>
+      </c>
+      <c r="AX32" s="4" t="inlineStr">
+        <is>
+          <t>Требует проверки</t>
+        </is>
+      </c>
+      <c r="AY32" s="3" t="inlineStr">
+        <is>
+          <t>Добавлено из портфеля для WAF/Anti-DDoS; KZ-дистрибьютора подтвердить вручную.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Imperva</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n"/>
+      <c r="C33" s="3" t="n"/>
+      <c r="D33" s="3" t="n"/>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="n"/>
+      <c r="G33" s="3" t="n"/>
+      <c r="H33" s="3" t="n"/>
+      <c r="I33" s="3" t="n"/>
+      <c r="J33" s="3" t="n"/>
+      <c r="K33" s="3" t="n"/>
+      <c r="L33" s="3" t="n"/>
+      <c r="M33" s="3" t="n"/>
+      <c r="N33" s="3" t="n"/>
+      <c r="O33" s="3" t="n"/>
+      <c r="P33" s="3" t="n"/>
+      <c r="Q33" s="3" t="n"/>
+      <c r="R33" s="3" t="n"/>
+      <c r="S33" s="3" t="n"/>
+      <c r="T33" s="3" t="n"/>
+      <c r="U33" s="3" t="n"/>
+      <c r="V33" s="3" t="n"/>
+      <c r="W33" s="3" t="n"/>
+      <c r="X33" s="3" t="n"/>
+      <c r="Y33" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="Z33" s="3" t="n"/>
+      <c r="AA33" s="3" t="n"/>
+      <c r="AB33" s="3" t="n"/>
+      <c r="AC33" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AD33" s="3" t="n"/>
+      <c r="AE33" s="3" t="n"/>
+      <c r="AF33" s="3" t="n"/>
+      <c r="AG33" s="3" t="n"/>
+      <c r="AH33" s="3" t="n"/>
+      <c r="AI33" s="3" t="n"/>
+      <c r="AJ33" s="3" t="n"/>
+      <c r="AK33" s="3" t="n"/>
+      <c r="AL33" s="3" t="n"/>
+      <c r="AM33" s="3" t="n"/>
+      <c r="AN33" s="3" t="n"/>
+      <c r="AO33" s="3" t="n"/>
+      <c r="AP33" s="3" t="n"/>
+      <c r="AQ33" s="3" t="n"/>
+      <c r="AR33" s="3" t="n"/>
+      <c r="AS33" s="3" t="n"/>
+      <c r="AT33" s="3" t="n"/>
+      <c r="AU33" s="3" t="n"/>
+      <c r="AV33" s="3" t="inlineStr">
+        <is>
+          <t>Softprom</t>
+        </is>
+      </c>
+      <c r="AW33" s="3" t="inlineStr">
+        <is>
+          <t>https://softprom.com/vendor/imperva ; https://www.imperva.com/products/data-security/unified-visibility/</t>
+        </is>
+      </c>
+      <c r="AX33" s="4" t="inlineStr">
+        <is>
+          <t>Подтверждено</t>
+        </is>
+      </c>
+      <c r="AY33" s="3" t="inlineStr">
+        <is>
+          <t>Imperva Data Security Fabric: защита, мониторинг и аудит доступа к базам данных; Softprom указывает официальный канал для Казахстана.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n"/>
+      <c r="C34" s="3" t="n"/>
+      <c r="D34" s="3" t="n"/>
+      <c r="E34" s="3" t="n"/>
+      <c r="F34" s="3" t="n"/>
+      <c r="G34" s="3" t="n"/>
+      <c r="H34" s="3" t="n"/>
+      <c r="I34" s="3" t="n"/>
+      <c r="J34" s="3" t="n"/>
+      <c r="K34" s="3" t="n"/>
+      <c r="L34" s="3" t="n"/>
+      <c r="M34" s="3" t="n"/>
+      <c r="N34" s="3" t="n"/>
+      <c r="O34" s="3" t="n"/>
+      <c r="P34" s="3" t="n"/>
+      <c r="Q34" s="3" t="n"/>
+      <c r="R34" s="3" t="n"/>
+      <c r="S34" s="3" t="n"/>
+      <c r="T34" s="3" t="n"/>
+      <c r="U34" s="3" t="n"/>
+      <c r="V34" s="3" t="n"/>
+      <c r="W34" s="3" t="n"/>
+      <c r="X34" s="3" t="n"/>
+      <c r="Y34" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="Z34" s="3" t="n"/>
+      <c r="AA34" s="3" t="n"/>
+      <c r="AB34" s="3" t="n"/>
+      <c r="AC34" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AD34" s="3" t="n"/>
+      <c r="AE34" s="3" t="n"/>
+      <c r="AF34" s="3" t="n"/>
+      <c r="AG34" s="3" t="n"/>
+      <c r="AH34" s="3" t="n"/>
+      <c r="AI34" s="3" t="n"/>
+      <c r="AJ34" s="3" t="n"/>
+      <c r="AK34" s="3" t="n"/>
+      <c r="AL34" s="3" t="n"/>
+      <c r="AM34" s="3" t="n"/>
+      <c r="AN34" s="3" t="n"/>
+      <c r="AO34" s="3" t="n"/>
+      <c r="AP34" s="3" t="n"/>
+      <c r="AQ34" s="3" t="n"/>
+      <c r="AR34" s="3" t="n"/>
+      <c r="AS34" s="3" t="n"/>
+      <c r="AT34" s="3" t="n"/>
+      <c r="AU34" s="3" t="n"/>
+      <c r="AV34" s="3" t="inlineStr">
+        <is>
+          <t>Не подтверждено; проверить через partner locator</t>
+        </is>
+      </c>
+      <c r="AW34" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cloudflare.com/partners/find-a-partner/</t>
+        </is>
+      </c>
+      <c r="AX34" s="4" t="inlineStr">
+        <is>
+          <t>Требует проверки</t>
+        </is>
+      </c>
+      <c r="AY34" s="3" t="inlineStr">
+        <is>
+          <t>Добавлено из портфеля для WAF/CDN/Anti-DDoS; KZ-дистрибьютора подтвердить вручную.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Radware</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n"/>
+      <c r="C35" s="3" t="n"/>
+      <c r="D35" s="3" t="n"/>
+      <c r="E35" s="3" t="n"/>
+      <c r="F35" s="3" t="n"/>
+      <c r="G35" s="3" t="n"/>
+      <c r="H35" s="3" t="n"/>
+      <c r="I35" s="3" t="n"/>
+      <c r="J35" s="3" t="n"/>
+      <c r="K35" s="3" t="n"/>
+      <c r="L35" s="3" t="n"/>
+      <c r="M35" s="3" t="n"/>
+      <c r="N35" s="3" t="n"/>
+      <c r="O35" s="3" t="n"/>
+      <c r="P35" s="3" t="n"/>
+      <c r="Q35" s="3" t="n"/>
+      <c r="R35" s="3" t="n"/>
+      <c r="S35" s="3" t="n"/>
+      <c r="T35" s="3" t="n"/>
+      <c r="U35" s="3" t="n"/>
+      <c r="V35" s="3" t="n"/>
+      <c r="W35" s="3" t="n"/>
+      <c r="X35" s="3" t="n"/>
+      <c r="Y35" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="Z35" s="3" t="n"/>
+      <c r="AA35" s="3" t="n"/>
+      <c r="AB35" s="3" t="n"/>
+      <c r="AC35" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AD35" s="3" t="n"/>
+      <c r="AE35" s="3" t="n"/>
+      <c r="AF35" s="3" t="n"/>
+      <c r="AG35" s="3" t="n"/>
+      <c r="AH35" s="3" t="n"/>
+      <c r="AI35" s="3" t="n"/>
+      <c r="AJ35" s="3" t="n"/>
+      <c r="AK35" s="3" t="n"/>
+      <c r="AL35" s="3" t="n"/>
+      <c r="AM35" s="3" t="n"/>
+      <c r="AN35" s="3" t="n"/>
+      <c r="AO35" s="3" t="n"/>
+      <c r="AP35" s="3" t="n"/>
+      <c r="AQ35" s="3" t="n"/>
+      <c r="AR35" s="3" t="n"/>
+      <c r="AS35" s="3" t="n"/>
+      <c r="AT35" s="3" t="n"/>
+      <c r="AU35" s="3" t="n"/>
+      <c r="AV35" s="3" t="inlineStr">
+        <is>
+          <t>MUK</t>
+        </is>
+      </c>
+      <c r="AW35" s="3" t="inlineStr">
+        <is>
+          <t>https://muk.group/ru/country/kz/</t>
+        </is>
+      </c>
+      <c r="AX35" s="4" t="inlineStr">
+        <is>
+          <t>Подтверждено</t>
+        </is>
+      </c>
+      <c r="AY35" s="3" t="inlineStr">
+        <is>
+          <t>MUK указывает Radware в действующем дистрибьюторском портфеле Казахстана.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>A10</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n"/>
+      <c r="C36" s="3" t="n"/>
+      <c r="D36" s="3" t="n"/>
+      <c r="E36" s="3" t="n"/>
+      <c r="F36" s="3" t="n"/>
+      <c r="G36" s="3" t="n"/>
+      <c r="H36" s="3" t="n"/>
+      <c r="I36" s="3" t="n"/>
+      <c r="J36" s="3" t="n"/>
+      <c r="K36" s="3" t="n"/>
+      <c r="L36" s="3" t="n"/>
+      <c r="M36" s="3" t="n"/>
+      <c r="N36" s="3" t="n"/>
+      <c r="O36" s="3" t="n"/>
+      <c r="P36" s="3" t="n"/>
+      <c r="Q36" s="3" t="n"/>
+      <c r="R36" s="3" t="n"/>
+      <c r="S36" s="3" t="n"/>
+      <c r="T36" s="3" t="n"/>
+      <c r="U36" s="3" t="n"/>
+      <c r="V36" s="3" t="n"/>
+      <c r="W36" s="3" t="n"/>
+      <c r="X36" s="3" t="n"/>
+      <c r="Y36" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="Z36" s="3" t="n"/>
+      <c r="AA36" s="3" t="n"/>
+      <c r="AB36" s="3" t="n"/>
+      <c r="AC36" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AD36" s="3" t="n"/>
+      <c r="AE36" s="3" t="n"/>
+      <c r="AF36" s="3" t="n"/>
+      <c r="AG36" s="3" t="n"/>
+      <c r="AH36" s="3" t="n"/>
+      <c r="AI36" s="3" t="n"/>
+      <c r="AJ36" s="3" t="n"/>
+      <c r="AK36" s="3" t="n"/>
+      <c r="AL36" s="3" t="n"/>
+      <c r="AM36" s="3" t="n"/>
+      <c r="AN36" s="3" t="n"/>
+      <c r="AO36" s="3" t="n"/>
+      <c r="AP36" s="3" t="n"/>
+      <c r="AQ36" s="3" t="n"/>
+      <c r="AR36" s="3" t="n"/>
+      <c r="AS36" s="3" t="n"/>
+      <c r="AT36" s="3" t="n"/>
+      <c r="AU36" s="3" t="n"/>
+      <c r="AV36" s="3" t="inlineStr">
+        <is>
+          <t>MUK; ASBIS Kazakhstan</t>
+        </is>
+      </c>
+      <c r="AW36" s="3" t="inlineStr">
+        <is>
+          <t>https://muk.group/ru/country/kz/ ; https://www.a10networks.com/partners/resellers/</t>
+        </is>
+      </c>
+      <c r="AX36" s="4" t="inlineStr">
+        <is>
+          <t>Подтверждено</t>
+        </is>
+      </c>
+      <c r="AY36" s="3" t="inlineStr">
+        <is>
+          <t>MUK указывает A10 в дистрибьюторском портфеле Казахстана; A10 Partner Locator указывает ASBIS KAZAKHSTAN TOO как Distributor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Barracuda</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n"/>
+      <c r="C37" s="3" t="n"/>
+      <c r="D37" s="3" t="n"/>
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="3" t="n"/>
+      <c r="G37" s="3" t="n"/>
+      <c r="H37" s="3" t="n"/>
+      <c r="I37" s="3" t="n"/>
+      <c r="J37" s="3" t="n"/>
+      <c r="K37" s="3" t="n"/>
+      <c r="L37" s="3" t="n"/>
+      <c r="M37" s="3" t="n"/>
+      <c r="N37" s="3" t="n"/>
+      <c r="O37" s="3" t="n"/>
+      <c r="P37" s="3" t="n"/>
+      <c r="Q37" s="3" t="n"/>
+      <c r="R37" s="3" t="n"/>
+      <c r="S37" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="T37" s="3" t="n"/>
+      <c r="U37" s="3" t="n"/>
+      <c r="V37" s="3" t="n"/>
+      <c r="W37" s="3" t="n"/>
+      <c r="X37" s="3" t="n"/>
+      <c r="Y37" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="Z37" s="3" t="n"/>
+      <c r="AA37" s="3" t="n"/>
+      <c r="AB37" s="3" t="n"/>
+      <c r="AC37" s="3" t="n"/>
+      <c r="AD37" s="3" t="n"/>
+      <c r="AE37" s="3" t="n"/>
+      <c r="AF37" s="3" t="n"/>
+      <c r="AG37" s="3" t="n"/>
+      <c r="AH37" s="3" t="n"/>
+      <c r="AI37" s="3" t="n"/>
+      <c r="AJ37" s="3" t="n"/>
+      <c r="AK37" s="3" t="n"/>
+      <c r="AL37" s="3" t="n"/>
+      <c r="AM37" s="3" t="n"/>
+      <c r="AN37" s="3" t="n"/>
+      <c r="AO37" s="3" t="n"/>
+      <c r="AP37" s="3" t="n"/>
+      <c r="AQ37" s="3" t="n"/>
+      <c r="AR37" s="3" t="n"/>
+      <c r="AS37" s="3" t="n"/>
+      <c r="AT37" s="3" t="n"/>
+      <c r="AU37" s="3" t="n"/>
+      <c r="AV37" s="3" t="inlineStr">
+        <is>
+          <t>Не подтверждено; проверить через partner locator</t>
+        </is>
+      </c>
+      <c r="AW37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.barracuda.com/partners</t>
+        </is>
+      </c>
+      <c r="AX37" s="4" t="inlineStr">
+        <is>
+          <t>Требует проверки</t>
+        </is>
+      </c>
+      <c r="AY37" s="3" t="inlineStr">
+        <is>
+          <t>Добавлено из портфеля для Email Security и WAF; KZ-дистрибьютора подтвердить вручную.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Axidian</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n"/>
+      <c r="C38" s="3" t="n"/>
+      <c r="D38" s="3" t="n"/>
+      <c r="E38" s="3" t="n"/>
+      <c r="F38" s="3" t="n"/>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="n"/>
+      <c r="J38" s="3" t="n"/>
+      <c r="K38" s="3" t="n"/>
+      <c r="L38" s="3" t="n"/>
+      <c r="M38" s="3" t="n"/>
+      <c r="N38" s="3" t="n"/>
+      <c r="O38" s="3" t="n"/>
+      <c r="P38" s="3" t="n"/>
+      <c r="Q38" s="3" t="n"/>
+      <c r="R38" s="3" t="n"/>
+      <c r="S38" s="3" t="n"/>
+      <c r="T38" s="3" t="n"/>
+      <c r="U38" s="3" t="n"/>
+      <c r="V38" s="3" t="n"/>
+      <c r="W38" s="3" t="n"/>
+      <c r="X38" s="3" t="n"/>
+      <c r="Y38" s="3" t="n"/>
+      <c r="Z38" s="3" t="n"/>
+      <c r="AA38" s="3" t="n"/>
+      <c r="AB38" s="3" t="n"/>
+      <c r="AC38" s="3" t="n"/>
+      <c r="AD38" s="3" t="n"/>
+      <c r="AE38" s="3" t="n"/>
+      <c r="AF38" s="3" t="n"/>
+      <c r="AG38" s="3" t="n"/>
+      <c r="AH38" s="3" t="n"/>
+      <c r="AI38" s="3" t="n"/>
+      <c r="AJ38" s="3" t="n"/>
+      <c r="AK38" s="3" t="n"/>
+      <c r="AL38" s="3" t="n"/>
+      <c r="AM38" s="3" t="n"/>
+      <c r="AN38" s="3" t="n"/>
+      <c r="AO38" s="3" t="n"/>
+      <c r="AP38" s="3" t="n"/>
+      <c r="AQ38" s="3" t="n"/>
+      <c r="AR38" s="3" t="n"/>
+      <c r="AS38" s="3" t="n"/>
+      <c r="AT38" s="3" t="n"/>
+      <c r="AU38" s="3" t="n"/>
+      <c r="AV38" s="3" t="inlineStr">
+        <is>
+          <t>MONT TECH</t>
+        </is>
+      </c>
+      <c r="AW38" s="3" t="inlineStr">
+        <is>
+          <t>https://monttech.kz/ru-kz/vendors</t>
+        </is>
+      </c>
+      <c r="AX38" s="4" t="inlineStr">
+        <is>
+          <t>Подтверждено</t>
+        </is>
+      </c>
+      <c r="AY38" s="3" t="inlineStr">
+        <is>
+          <t>Axidian присутствует в актуальном портфеле MONT TECH Казахстан, включая решения MFA и PAM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Fudo</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n"/>
+      <c r="C39" s="3" t="n"/>
+      <c r="D39" s="3" t="n"/>
+      <c r="E39" s="3" t="n"/>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="n"/>
+      <c r="H39" s="3" t="n"/>
+      <c r="I39" s="3" t="n"/>
+      <c r="J39" s="3" t="n"/>
+      <c r="K39" s="3" t="n"/>
+      <c r="L39" s="3" t="n"/>
+      <c r="M39" s="3" t="n"/>
+      <c r="N39" s="3" t="n"/>
+      <c r="O39" s="3" t="n"/>
+      <c r="P39" s="3" t="n"/>
+      <c r="Q39" s="3" t="n"/>
+      <c r="R39" s="3" t="n"/>
+      <c r="S39" s="3" t="n"/>
+      <c r="T39" s="3" t="n"/>
+      <c r="U39" s="3" t="n"/>
+      <c r="V39" s="3" t="n"/>
+      <c r="W39" s="3" t="n"/>
+      <c r="X39" s="3" t="n"/>
+      <c r="Y39" s="3" t="n"/>
+      <c r="Z39" s="3" t="n"/>
+      <c r="AA39" s="3" t="n"/>
+      <c r="AB39" s="3" t="n"/>
+      <c r="AC39" s="3" t="n"/>
+      <c r="AD39" s="3" t="n"/>
+      <c r="AE39" s="3" t="n"/>
+      <c r="AF39" s="3" t="n"/>
+      <c r="AG39" s="3" t="n"/>
+      <c r="AH39" s="3" t="n"/>
+      <c r="AI39" s="3" t="n"/>
+      <c r="AJ39" s="3" t="n"/>
+      <c r="AK39" s="3" t="n"/>
+      <c r="AL39" s="3" t="n"/>
+      <c r="AM39" s="3" t="n"/>
+      <c r="AN39" s="3" t="n"/>
+      <c r="AO39" s="3" t="n"/>
+      <c r="AP39" s="3" t="n"/>
+      <c r="AQ39" s="3" t="n"/>
+      <c r="AR39" s="3" t="n"/>
+      <c r="AS39" s="3" t="n"/>
+      <c r="AT39" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AU39" s="3" t="n"/>
+      <c r="AV39" s="3" t="inlineStr">
+        <is>
+          <t>Не подтверждено; проверить через partner locator</t>
+        </is>
+      </c>
+      <c r="AW39" s="3" t="inlineStr">
+        <is>
+          <t>https://fudosecurity.com/partners/</t>
+        </is>
+      </c>
+      <c r="AX39" s="4" t="inlineStr">
+        <is>
+          <t>Требует проверки</t>
+        </is>
+      </c>
+      <c r="AY39" s="3" t="inlineStr">
+        <is>
+          <t>Добавлено из портфеля для PAM/session management; KZ-дистрибьютора подтвердить вручную.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>HCL AppScan</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n"/>
+      <c r="C40" s="3" t="n"/>
+      <c r="D40" s="3" t="n"/>
+      <c r="E40" s="3" t="n"/>
+      <c r="F40" s="3" t="n"/>
+      <c r="G40" s="3" t="n"/>
+      <c r="H40" s="3" t="n"/>
+      <c r="I40" s="3" t="n"/>
+      <c r="J40" s="3" t="n"/>
+      <c r="K40" s="3" t="n"/>
+      <c r="L40" s="3" t="n"/>
+      <c r="M40" s="3" t="n"/>
+      <c r="N40" s="3" t="n"/>
+      <c r="O40" s="3" t="n"/>
+      <c r="P40" s="3" t="n"/>
+      <c r="Q40" s="3" t="n"/>
+      <c r="R40" s="3" t="n"/>
+      <c r="S40" s="3" t="n"/>
+      <c r="T40" s="3" t="n"/>
+      <c r="U40" s="3" t="n"/>
+      <c r="V40" s="3" t="n"/>
+      <c r="W40" s="3" t="n"/>
+      <c r="X40" s="3" t="n"/>
+      <c r="Y40" s="3" t="n"/>
+      <c r="Z40" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AA40" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AB40" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AC40" s="3" t="n"/>
+      <c r="AD40" s="3" t="n"/>
+      <c r="AE40" s="3" t="n"/>
+      <c r="AF40" s="3" t="n"/>
+      <c r="AG40" s="3" t="n"/>
+      <c r="AH40" s="3" t="n"/>
+      <c r="AI40" s="3" t="n"/>
+      <c r="AJ40" s="3" t="n"/>
+      <c r="AK40" s="3" t="n"/>
+      <c r="AL40" s="3" t="n"/>
+      <c r="AM40" s="3" t="n"/>
+      <c r="AN40" s="3" t="n"/>
+      <c r="AO40" s="3" t="n"/>
+      <c r="AP40" s="3" t="n"/>
+      <c r="AQ40" s="3" t="n"/>
+      <c r="AR40" s="3" t="n"/>
+      <c r="AS40" s="3" t="n"/>
+      <c r="AT40" s="3" t="n"/>
+      <c r="AU40" s="3" t="n"/>
+      <c r="AV40" s="3" t="inlineStr">
+        <is>
+          <t>MONT TECH; MUK</t>
+        </is>
+      </c>
+      <c r="AW40" s="3" t="inlineStr">
+        <is>
+          <t>https://monttech.kz/ru-kz/vendors ; https://muk.group/ru/country/kz/</t>
+        </is>
+      </c>
+      <c r="AX40" s="4" t="inlineStr">
+        <is>
+          <t>Подтверждено</t>
+        </is>
+      </c>
+      <c r="AY40" s="3" t="inlineStr">
+        <is>
+          <t>HCLSoftware присутствует в актуальных портфелях MONT TECH и MUK Казахстан; AppScan относится к линейке HCLSoftware.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Positive Technologies</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n"/>
+      <c r="C41" s="3" t="n"/>
+      <c r="D41" s="3" t="n"/>
+      <c r="E41" s="3" t="n"/>
+      <c r="F41" s="3" t="n"/>
+      <c r="G41" s="3" t="n"/>
+      <c r="H41" s="3" t="n"/>
+      <c r="I41" s="3" t="n"/>
+      <c r="J41" s="3" t="n"/>
+      <c r="K41" s="3" t="n"/>
+      <c r="L41" s="3" t="n"/>
+      <c r="M41" s="3" t="n"/>
+      <c r="N41" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="O41" s="3" t="n"/>
+      <c r="P41" s="3" t="n"/>
+      <c r="Q41" s="3" t="n"/>
+      <c r="R41" s="3" t="n"/>
+      <c r="S41" s="3" t="n"/>
+      <c r="T41" s="3" t="n"/>
+      <c r="U41" s="3" t="n"/>
+      <c r="V41" s="3" t="n"/>
+      <c r="W41" s="3" t="n"/>
+      <c r="X41" s="3" t="n"/>
+      <c r="Y41" s="3" t="n"/>
+      <c r="Z41" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AA41" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AB41" s="3" t="n"/>
+      <c r="AC41" s="3" t="n"/>
+      <c r="AD41" s="3" t="n"/>
+      <c r="AE41" s="3" t="n"/>
+      <c r="AF41" s="3" t="n"/>
+      <c r="AG41" s="3" t="n"/>
+      <c r="AH41" s="3" t="n"/>
+      <c r="AI41" s="3" t="n"/>
+      <c r="AJ41" s="3" t="n"/>
+      <c r="AK41" s="3" t="n"/>
+      <c r="AL41" s="3" t="n"/>
+      <c r="AM41" s="3" t="n"/>
+      <c r="AN41" s="3" t="n"/>
+      <c r="AO41" s="3" t="n"/>
+      <c r="AP41" s="3" t="n"/>
+      <c r="AQ41" s="3" t="n"/>
+      <c r="AR41" s="3" t="n"/>
+      <c r="AS41" s="3" t="n"/>
+      <c r="AT41" s="3" t="n"/>
+      <c r="AU41" s="3" t="n"/>
+      <c r="AV41" s="3" t="inlineStr">
+        <is>
+          <t>MONT TECH</t>
+        </is>
+      </c>
+      <c r="AW41" s="3" t="inlineStr">
+        <is>
+          <t>https://monttech.kz/ru-kz/vendors</t>
+        </is>
+      </c>
+      <c r="AX41" s="4" t="inlineStr">
+        <is>
+          <t>Подтверждено</t>
+        </is>
+      </c>
+      <c r="AY41" s="3" t="inlineStr">
+        <is>
+          <t>Positive Technologies присутствует в актуальном портфеле MONT TECH Казахстан для VM, AppSec, SIEM и WAF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>R-Vision SIEM</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n"/>
+      <c r="C42" s="3" t="n"/>
+      <c r="D42" s="3" t="n"/>
+      <c r="E42" s="3" t="n"/>
+      <c r="F42" s="3" t="n"/>
+      <c r="G42" s="3" t="n"/>
+      <c r="H42" s="3" t="n"/>
+      <c r="I42" s="3" t="n"/>
+      <c r="J42" s="3" t="n"/>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="L42" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="M42" s="3" t="n"/>
+      <c r="N42" s="3" t="n"/>
+      <c r="O42" s="3" t="n"/>
+      <c r="P42" s="3" t="n"/>
+      <c r="Q42" s="3" t="n"/>
+      <c r="R42" s="3" t="n"/>
+      <c r="S42" s="3" t="n"/>
+      <c r="T42" s="3" t="n"/>
+      <c r="U42" s="3" t="n"/>
+      <c r="V42" s="3" t="n"/>
+      <c r="W42" s="3" t="n"/>
+      <c r="X42" s="3" t="n"/>
+      <c r="Y42" s="3" t="n"/>
+      <c r="Z42" s="3" t="n"/>
+      <c r="AA42" s="3" t="n"/>
+      <c r="AB42" s="3" t="n"/>
+      <c r="AC42" s="3" t="n"/>
+      <c r="AD42" s="3" t="n"/>
+      <c r="AE42" s="3" t="n"/>
+      <c r="AF42" s="3" t="n"/>
+      <c r="AG42" s="3" t="n"/>
+      <c r="AH42" s="3" t="n"/>
+      <c r="AI42" s="3" t="n"/>
+      <c r="AJ42" s="3" t="n"/>
+      <c r="AK42" s="3" t="n"/>
+      <c r="AL42" s="3" t="n"/>
+      <c r="AM42" s="3" t="n"/>
+      <c r="AN42" s="3" t="n"/>
+      <c r="AO42" s="3" t="n"/>
+      <c r="AP42" s="3" t="n"/>
+      <c r="AQ42" s="3" t="n"/>
+      <c r="AR42" s="3" t="n"/>
+      <c r="AS42" s="3" t="n"/>
+      <c r="AT42" s="3" t="n"/>
+      <c r="AU42" s="3" t="n"/>
+      <c r="AV42" s="3" t="inlineStr">
+        <is>
+          <t>MONT TECH</t>
+        </is>
+      </c>
+      <c r="AW42" s="3" t="inlineStr">
+        <is>
+          <t>https://monttech.kz/ru-kz/vendors</t>
+        </is>
+      </c>
+      <c r="AX42" s="4" t="inlineStr">
+        <is>
+          <t>Подтверждено</t>
+        </is>
+      </c>
+      <c r="AY42" s="3" t="inlineStr">
+        <is>
+          <t>R-Vision присутствует в актуальном портфеле MONT TECH Казахстан для SIEM, SOAR и UEBA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>QazSIEM</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n"/>
+      <c r="C43" s="3" t="n"/>
+      <c r="D43" s="3" t="n"/>
+      <c r="E43" s="3" t="n"/>
+      <c r="F43" s="3" t="n"/>
+      <c r="G43" s="3" t="n"/>
+      <c r="H43" s="3" t="n"/>
+      <c r="I43" s="3" t="n"/>
+      <c r="J43" s="3" t="n"/>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="n"/>
+      <c r="M43" s="3" t="n"/>
+      <c r="N43" s="3" t="n"/>
+      <c r="O43" s="3" t="n"/>
+      <c r="P43" s="3" t="n"/>
+      <c r="Q43" s="3" t="n"/>
+      <c r="R43" s="3" t="n"/>
+      <c r="S43" s="3" t="n"/>
+      <c r="T43" s="3" t="n"/>
+      <c r="U43" s="3" t="n"/>
+      <c r="V43" s="3" t="n"/>
+      <c r="W43" s="3" t="n"/>
+      <c r="X43" s="3" t="n"/>
+      <c r="Y43" s="3" t="n"/>
+      <c r="Z43" s="3" t="n"/>
+      <c r="AA43" s="3" t="n"/>
+      <c r="AB43" s="3" t="n"/>
+      <c r="AC43" s="3" t="n"/>
+      <c r="AD43" s="3" t="n"/>
+      <c r="AE43" s="3" t="n"/>
+      <c r="AF43" s="3" t="n"/>
+      <c r="AG43" s="3" t="n"/>
+      <c r="AH43" s="3" t="n"/>
+      <c r="AI43" s="3" t="n"/>
+      <c r="AJ43" s="3" t="n"/>
+      <c r="AK43" s="3" t="n"/>
+      <c r="AL43" s="3" t="n"/>
+      <c r="AM43" s="3" t="n"/>
+      <c r="AN43" s="3" t="n"/>
+      <c r="AO43" s="3" t="n"/>
+      <c r="AP43" s="3" t="n"/>
+      <c r="AQ43" s="3" t="n"/>
+      <c r="AR43" s="3" t="n"/>
+      <c r="AS43" s="3" t="n"/>
+      <c r="AT43" s="3" t="n"/>
+      <c r="AU43" s="3" t="n"/>
+      <c r="AV43" s="3" t="inlineStr">
+        <is>
+          <t>Не подтверждено; проверить через partner locator</t>
+        </is>
+      </c>
+      <c r="AW43" s="3" t="inlineStr">
+        <is>
+          <t>https://qazsiem.kz/</t>
+        </is>
+      </c>
+      <c r="AX43" s="4" t="inlineStr">
+        <is>
+          <t>Требует проверки</t>
+        </is>
+      </c>
+      <c r="AY43" s="3" t="inlineStr">
+        <is>
+          <t>Добавлено из портфеля для SIEM; KZ-дистрибьютора подтвердить вручную.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Garda Technologies (Гарда)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AV44" t="inlineStr">
+        <is>
+          <t>Axoft Kazakhstan</t>
+        </is>
+      </c>
+      <c r="AW44" t="inlineStr">
+        <is>
+          <t>https://axoftglobal.com/en-kz/vendors/garda ; https://garda.ai/products/data-protection/dbf</t>
+        </is>
+      </c>
+      <c r="AX44" t="inlineStr">
+        <is>
+          <t>Подтверждено</t>
+        </is>
+      </c>
+      <c r="AY44" t="inlineStr">
+        <is>
+          <t>Гарда DBF: централизованная защита баз данных, аудит операций и блокировка нелегитимных запросов; вендор представлен в портфеле Axoft Kazakhstan.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
@@ -3239,7 +4370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3922,8 +5053,52 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Imperva</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Softprom</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://softprom.com/vendor/imperva ; https://www.imperva.com/products/data-security/unified-visibility/</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Подтверждено. Imperva DSF обеспечивает мониторинг, аудит и защиту доступа к базам данных; Softprom указывает официальный канал для Казахстана.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Garda Technologies (Гарда)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Axoft Kazakhstan</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://axoftglobal.com/en-kz/vendors/garda ; https://garda.ai/products/data-protection/dbf</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Подтверждено. Гарда DBF защищает базы данных; вендор представлен в портфеле Axoft Kazakhstan.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>

</xml_diff>